<commit_message>
Se ajusto codigo de farmatodo para corrida
</commit_message>
<xml_diff>
--- a/app/Archivos/Template/Template_HRC_farmatodo.xlsx
+++ b/app/Archivos/Template/Template_HRC_farmatodo.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -673,7 +673,7 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="64" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -718,7 +718,7 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>218819138.28</v>
+        <v>218819139.43</v>
       </c>
     </row>
     <row r="7">
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>218819138.28</v>
+        <v>218819139.43</v>
       </c>
     </row>
     <row r="8">
@@ -781,7 +781,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9/18/25</t>
+          <t>#m/#d/25</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>218819138.28</v>
+        <v>218819139.43</v>
       </c>
     </row>
     <row r="13"/>
@@ -838,12 +838,12 @@
     <row r="19">
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Nota Debito</t>
+          <t>Factura</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>‭PMP1279547‬</t>
+          <t>PMP1279547</t>
         </is>
       </c>
       <c r="E19" s="6" t="n">
@@ -854,21 +854,17 @@
       <c r="H19" s="6" t="n">
         <v>126062332.48</v>
       </c>
-      <c r="I19" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> ‭PMP1279547‬</t>
-        </is>
-      </c>
+      <c r="I19" s="11" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Nota Debito</t>
+          <t>Factura</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>‭PMP1279567‬</t>
+          <t>PMP1279567</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
@@ -879,21 +875,17 @@
       <c r="H20" s="6" t="n">
         <v>93147129.05</v>
       </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> ‭PMP1279567‬</t>
-        </is>
-      </c>
+      <c r="I20" s="11" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Nota Debito</t>
+          <t>Factura</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>‭PMP1279890‬</t>
+          <t>PMP1279890</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
@@ -904,11 +896,7 @@
       <c r="H21" s="6" t="n">
         <v>3344306.86</v>
       </c>
-      <c r="I21" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> ‭PMP1279890‬</t>
-        </is>
-      </c>
+      <c r="I21" s="11" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="C22" s="10" t="inlineStr">
@@ -918,20 +906,28 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>‭NC-PMP1279547‬</t>
+          <t>PMP1279547</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
         <v>-2118694.66</v>
       </c>
-      <c r="F22" s="10" t="inlineStr"/>
-      <c r="G22" s="10" t="inlineStr"/>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>DPP</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
       <c r="H22" s="6" t="n">
         <v>-2118694.66</v>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ‭NC-PMP1279547‬</t>
+          <t>DPP PMP1279547 OC:14007431 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
         </is>
       </c>
     </row>
@@ -943,20 +939,28 @@
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>‭NC-PMP1279567‬</t>
+          <t>PMP1279567</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
         <v>-1565497.97</v>
       </c>
-      <c r="F23" s="10" t="inlineStr"/>
-      <c r="G23" s="10" t="inlineStr"/>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>DPP</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
       <c r="H23" s="6" t="n">
         <v>-1565497.97</v>
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ‭NC-PMP1279567‬</t>
+          <t>DPP PMP1279567 OC:14007453 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
         </is>
       </c>
     </row>
@@ -968,72 +972,127 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>‭NC-PMP1279890‬</t>
+          <t>PMP1279890</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
         <v>-50437.48</v>
       </c>
-      <c r="F24" s="10" t="inlineStr"/>
-      <c r="G24" s="10" t="inlineStr"/>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>DPP</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
       <c r="H24" s="6" t="n">
         <v>-50437.48</v>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ‭NC-PMP1279890‬</t>
+          <t>DPP PMP1279890 OC:14007449 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="10" t="inlineStr"/>
-      <c r="D25" s="10" t="inlineStr"/>
-      <c r="E25" s="6" t="inlineStr"/>
-      <c r="F25" s="10" t="inlineStr"/>
-      <c r="G25" s="10" t="inlineStr"/>
-      <c r="H25" s="6" t="inlineStr"/>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos no asociados a FC</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>PMP1279547</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>0.7000000029802322</v>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>0.7000000029802322</v>
+      </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t> </t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="C26" s="10" t="inlineStr"/>
-      <c r="D26" s="10" t="inlineStr"/>
-      <c r="E26" s="6" t="inlineStr"/>
-      <c r="F26" s="10" t="inlineStr"/>
-      <c r="G26" s="10" t="inlineStr"/>
-      <c r="H26" s="6" t="inlineStr"/>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos no asociados a FC</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>PMP1279567</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>0.3100000023841858</v>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>0.3100000023841858</v>
+      </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t> </t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="C27" s="10" t="inlineStr"/>
-      <c r="D27" s="10" t="inlineStr"/>
-      <c r="E27" s="6" t="inlineStr"/>
-      <c r="F27" s="10" t="inlineStr"/>
-      <c r="G27" s="10" t="inlineStr"/>
-      <c r="H27" s="6" t="inlineStr"/>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos no asociados a FC</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>PMP1279890</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>0.1400000001303852</v>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>0.1400000001303852</v>
+      </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="C28" s="10" t="inlineStr"/>
-      <c r="D28" s="10" t="inlineStr"/>
-      <c r="E28" s="6" t="inlineStr"/>
-      <c r="F28" s="10" t="inlineStr"/>
-      <c r="G28" s="10" t="inlineStr"/>
-      <c r="H28" s="6" t="inlineStr"/>
-      <c r="I28" s="11" t="inlineStr">
-        <is>
-          <t> </t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
     </row>

</xml_diff>